<commit_message>
📊 [auto] Economic data update — 2026-09-01 17:15 UTC
</commit_message>
<xml_diff>
--- a/reports/excel/MacroPulse_2026-09-01.xlsx
+++ b/reports/excel/MacroPulse_2026-09-01.xlsx
@@ -651,7 +651,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-09-01 01:21 UTC</t>
+          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-09-01 17:15 UTC</t>
         </is>
       </c>
     </row>
@@ -1732,12 +1732,12 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>7,359</t>
+          <t>7,271</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>2.15%</t>
+          <t>2.57%</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>-2.36%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🔥 通膨指標　歷史數據　　生成時間：2026-09-01 01:21 UTC</t>
+          <t>🔥 通膨指標　歷史數據　　生成時間：2026-09-01 17:15 UTC</t>
         </is>
       </c>
     </row>
@@ -14688,7 +14688,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>📈 經濟成長　歷史數據　　生成時間：2026-09-01 01:21 UTC</t>
+          <t>📈 經濟成長　歷史數據　　生成時間：2026-09-01 17:15 UTC</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>👷 勞動市場　歷史數據　　生成時間：2026-09-01 01:21 UTC</t>
+          <t>👷 勞動市場　歷史數據　　生成時間：2026-09-01 17:15 UTC</t>
         </is>
       </c>
     </row>
@@ -35195,17 +35195,17 @@
       </c>
       <c r="Q110" s="19" t="inlineStr">
         <is>
-          <t>7,359</t>
+          <t>7,182</t>
         </is>
       </c>
       <c r="R110" s="19" t="inlineStr">
         <is>
-          <t>2.15%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="S110" s="19" t="inlineStr">
         <is>
-          <t>-2.36%</t>
+          <t>-4.71%</t>
         </is>
       </c>
     </row>
@@ -35680,17 +35680,17 @@
       </c>
       <c r="Q115" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>7,271</t>
         </is>
       </c>
       <c r="R115" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2.57%</t>
         </is>
       </c>
       <c r="S115" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1.24%</t>
         </is>
       </c>
     </row>
@@ -36517,7 +36517,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏦 利率與債券　歷史數據　　生成時間：2026-09-01 01:21 UTC</t>
+          <t>🏦 利率與債券　歷史數據　　生成時間：2026-09-01 17:15 UTC</t>
         </is>
       </c>
     </row>
@@ -48336,7 +48336,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>💭 信心指數　歷史數據　　生成時間：2026-09-01 01:21 UTC</t>
+          <t>💭 信心指數　歷史數據　　生成時間：2026-09-01 17:15 UTC</t>
         </is>
       </c>
     </row>
@@ -56513,7 +56513,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-09-01 01:21 UTC</t>
+          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-09-01 17:15 UTC</t>
         </is>
       </c>
     </row>
@@ -59729,7 +59729,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏠 房市　歷史數據　　生成時間：2026-09-01 01:21 UTC</t>
+          <t>🏠 房市　歷史數據　　生成時間：2026-09-01 17:15 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>